<commit_message>
feat: Add Encuesta dashboard with survey data visualization
- Implemented a new Encuesta dashboard page using React and Recharts for visualizing survey responses.
- Added a custom tooltip for pie chart segments displaying detailed information about responses.
- Introduced loading state with skeleton components for better user experience during data fetching.
- Created a Python script to check columns in the survey Excel file.
- Added a script to remove responses from "Capital Economics" and recalculate statistics.
- Implemented a verification script to ensure "Capital Economics" responses are removed from the dataset.
</commit_message>
<xml_diff>
--- a/Encuesta Mario.xlsx
+++ b/Encuesta Mario.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\David Ricardo\Desktop\FLAR\Secular forum\Secular_Hub_App\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE1D035B-C644-49CD-9D39-47F3C063A982}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45E31659-8CBA-40DF-B8BA-33AF9E123C88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$C$651</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$C$427</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -123,9 +123,6 @@
     <t>No</t>
   </si>
   <si>
-    <t>Numero</t>
-  </si>
-  <si>
     <t>"Downside risks include labour market weakness spilling over to consumer spending, foreshadowing a recession, with stagflationary dynamics amplified by tariff aftershocks" y "As markets begin to recognise that valuations of AI and related technologies may already reflect their true earnings potential, a normalisation phase could follow" y "The Fed's reaction function has become more dovish...but its institutional independence may be tested by legal challenges and political pressure."</t>
   </si>
   <si>
@@ -205,6 +202,9 @@
   </si>
   <si>
     <t>Fidelity International</t>
+  </si>
+  <si>
+    <t>Pregunta</t>
   </si>
 </sst>
 </file>
@@ -394,30 +394,30 @@
   </cellStyleXfs>
   <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment readingOrder="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -735,6 +735,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:G651"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -751,21 +752,21 @@
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C2" s="3">
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>4</v>
       </c>
@@ -776,40 +777,40 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>4</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C4" s="3">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>4</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C5" s="3">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>4</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C6" s="3">
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>4</v>
       </c>
@@ -821,45 +822,45 @@
       </c>
       <c r="D7" s="4"/>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>4</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C8" s="3">
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>4</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C9" s="3">
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>4</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C10" s="3">
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>4</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C11" s="3">
         <v>9</v>
@@ -870,24 +871,24 @@
         <v>4</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C12" s="3">
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>4</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C13" s="3">
         <v>11</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>4</v>
       </c>
@@ -898,7 +899,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>4</v>
       </c>
@@ -909,7 +910,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>4</v>
       </c>
@@ -920,7 +921,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>4</v>
       </c>
@@ -931,7 +932,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>4</v>
       </c>
@@ -942,7 +943,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>4</v>
       </c>
@@ -953,7 +954,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
         <v>4</v>
       </c>
@@ -964,7 +965,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
         <v>4</v>
       </c>
@@ -975,18 +976,18 @@
         <v>29</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
         <v>4</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C22" s="3">
         <v>14</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
         <v>4</v>
       </c>
@@ -997,7 +998,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
         <v>4</v>
       </c>
@@ -1008,84 +1009,84 @@
         <v>16</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
         <v>4</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C25" s="3">
         <v>17</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
         <v>4</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C26" s="3">
         <v>18</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
         <v>4</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C27" s="3">
         <v>19</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
         <v>17</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C28" s="3">
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
         <v>17</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C29" s="3">
         <v>2</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
         <v>17</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C30" s="3">
         <v>3</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
         <v>17</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C31" s="3">
         <v>4</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
         <v>17</v>
       </c>
@@ -1096,45 +1097,45 @@
         <v>5</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" s="3" t="s">
         <v>17</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C33" s="3">
         <v>6</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
         <v>17</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C34" s="3">
         <v>7</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" s="3" t="s">
         <v>17</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C35" s="3">
         <v>8</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" s="3" t="s">
         <v>17</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C36" s="3">
         <v>9</v>
@@ -1145,24 +1146,24 @@
         <v>17</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C37" s="3">
         <v>10</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38" s="3" t="s">
         <v>17</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C38" s="3">
         <v>11</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
         <v>17</v>
       </c>
@@ -1173,7 +1174,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40" s="3" t="s">
         <v>17</v>
       </c>
@@ -1184,7 +1185,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
         <v>17</v>
       </c>
@@ -1195,7 +1196,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" s="3" t="s">
         <v>17</v>
       </c>
@@ -1206,7 +1207,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" s="3" t="s">
         <v>17</v>
       </c>
@@ -1217,7 +1218,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44" s="3" t="s">
         <v>17</v>
       </c>
@@ -1228,7 +1229,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" s="3" t="s">
         <v>17</v>
       </c>
@@ -1239,7 +1240,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A46" s="3" t="s">
         <v>17</v>
       </c>
@@ -1250,7 +1251,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" s="3" t="s">
         <v>17</v>
       </c>
@@ -1261,7 +1262,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48" s="3" t="s">
         <v>17</v>
       </c>
@@ -1272,95 +1273,95 @@
         <v>15</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" s="3" t="s">
         <v>17</v>
       </c>
       <c r="B49" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C49" s="3">
         <v>16</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" s="3" t="s">
         <v>17</v>
       </c>
       <c r="B50" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C50" s="3">
         <v>17</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51" s="3" t="s">
         <v>17</v>
       </c>
       <c r="B51" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C51" s="3">
         <v>18</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52" s="3" t="s">
         <v>17</v>
       </c>
       <c r="B52" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C52" s="3">
         <v>19</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53" s="3" t="s">
         <v>5</v>
       </c>
       <c r="B53" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C53" s="3">
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54" s="3" t="s">
         <v>5</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C54" s="3">
         <v>2</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55" s="3" t="s">
         <v>5</v>
       </c>
       <c r="B55" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C55" s="3">
         <v>3</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
         <v>5</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C56" s="3">
         <v>4</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A57" s="3" t="s">
         <v>5</v>
       </c>
@@ -1371,45 +1372,45 @@
         <v>5</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A58" s="3" t="s">
         <v>5</v>
       </c>
       <c r="B58" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C58" s="3">
         <v>6</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A59" s="3" t="s">
         <v>5</v>
       </c>
       <c r="B59" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C59" s="3">
         <v>7</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60" s="3" t="s">
         <v>5</v>
       </c>
       <c r="B60" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C60" s="3">
         <v>8</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A61" s="3" t="s">
         <v>5</v>
       </c>
       <c r="B61" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C61" s="3">
         <v>9</v>
@@ -1420,24 +1421,24 @@
         <v>5</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C62" s="3">
         <v>10</v>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A63" s="3" t="s">
         <v>5</v>
       </c>
       <c r="B63" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C63" s="3">
         <v>11</v>
       </c>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A64" s="3" t="s">
         <v>5</v>
       </c>
@@ -1448,7 +1449,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A65" s="3" t="s">
         <v>5</v>
       </c>
@@ -1459,7 +1460,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A66" s="3" t="s">
         <v>5</v>
       </c>
@@ -1470,7 +1471,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A67" s="3" t="s">
         <v>5</v>
       </c>
@@ -1481,7 +1482,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A68" s="3" t="s">
         <v>5</v>
       </c>
@@ -1492,7 +1493,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A69" s="3" t="s">
         <v>5</v>
       </c>
@@ -1503,7 +1504,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A70" s="3" t="s">
         <v>5</v>
       </c>
@@ -1514,7 +1515,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A71" s="3" t="s">
         <v>5</v>
       </c>
@@ -1525,7 +1526,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A72" s="3" t="s">
         <v>5</v>
       </c>
@@ -1536,7 +1537,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A73" s="3" t="s">
         <v>5</v>
       </c>
@@ -1547,7 +1548,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A74" s="3" t="s">
         <v>5</v>
       </c>
@@ -1558,7 +1559,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A75" s="3" t="s">
         <v>5</v>
       </c>
@@ -1569,51 +1570,51 @@
         <v>17</v>
       </c>
     </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A76" s="3" t="s">
         <v>5</v>
       </c>
       <c r="B76" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C76" s="3">
         <v>18</v>
       </c>
     </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A77" s="3" t="s">
         <v>5</v>
       </c>
       <c r="B77" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C77" s="3">
         <v>19</v>
       </c>
     </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A78" s="3" t="s">
         <v>16</v>
       </c>
       <c r="B78" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C78" s="3">
         <v>1</v>
       </c>
     </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A79" s="3" t="s">
         <v>16</v>
       </c>
       <c r="B79" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C79" s="3">
         <v>2</v>
       </c>
     </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A80" s="3" t="s">
         <v>16</v>
       </c>
@@ -1624,7 +1625,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A81" s="3" t="s">
         <v>16</v>
       </c>
@@ -1635,7 +1636,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A82" s="3" t="s">
         <v>16</v>
       </c>
@@ -1646,45 +1647,45 @@
         <v>5</v>
       </c>
     </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A83" s="3" t="s">
         <v>16</v>
       </c>
       <c r="B83" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C83" s="3">
         <v>6</v>
       </c>
     </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A84" s="3" t="s">
         <v>16</v>
       </c>
       <c r="B84" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C84" s="3">
         <v>7</v>
       </c>
     </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A85" s="3" t="s">
         <v>16</v>
       </c>
       <c r="B85" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C85" s="3">
         <v>8</v>
       </c>
     </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A86" s="3" t="s">
         <v>16</v>
       </c>
       <c r="B86" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C86" s="3">
         <v>9</v>
@@ -1695,24 +1696,24 @@
         <v>16</v>
       </c>
       <c r="B87" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C87" s="3">
         <v>10</v>
       </c>
     </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A88" s="3" t="s">
         <v>16</v>
       </c>
       <c r="B88" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C88" s="3">
         <v>11</v>
       </c>
     </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A89" s="3" t="s">
         <v>16</v>
       </c>
@@ -1723,7 +1724,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A90" s="3" t="s">
         <v>16</v>
       </c>
@@ -1734,7 +1735,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A91" s="3" t="s">
         <v>16</v>
       </c>
@@ -1745,7 +1746,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A92" s="3" t="s">
         <v>16</v>
       </c>
@@ -1756,7 +1757,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A93" s="3" t="s">
         <v>16</v>
       </c>
@@ -1767,7 +1768,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A94" s="3" t="s">
         <v>16</v>
       </c>
@@ -1778,7 +1779,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A95" s="3" t="s">
         <v>16</v>
       </c>
@@ -1789,7 +1790,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A96" s="3" t="s">
         <v>16</v>
       </c>
@@ -1800,7 +1801,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A97" s="3" t="s">
         <v>16</v>
       </c>
@@ -1811,7 +1812,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A98" s="3" t="s">
         <v>16</v>
       </c>
@@ -1822,7 +1823,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A99" s="3" t="s">
         <v>16</v>
       </c>
@@ -1833,18 +1834,18 @@
         <v>16</v>
       </c>
     </row>
-    <row r="100" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A100" s="3" t="s">
         <v>16</v>
       </c>
       <c r="B100" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C100" s="3">
         <v>17</v>
       </c>
     </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A101" s="3" t="s">
         <v>16</v>
       </c>
@@ -1855,18 +1856,18 @@
         <v>18</v>
       </c>
     </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A102" s="3" t="s">
         <v>16</v>
       </c>
       <c r="B102" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C102" s="3">
         <v>19</v>
       </c>
     </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A103" s="3" t="s">
         <v>6</v>
       </c>
@@ -1877,29 +1878,29 @@
         <v>1</v>
       </c>
     </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A104" s="3" t="s">
         <v>6</v>
       </c>
       <c r="B104" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C104" s="3">
         <v>2</v>
       </c>
     </row>
-    <row r="105" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A105" s="3" t="s">
         <v>6</v>
       </c>
       <c r="B105" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C105" s="3">
         <v>3</v>
       </c>
     </row>
-    <row r="106" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A106" s="3" t="s">
         <v>6</v>
       </c>
@@ -1910,7 +1911,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="107" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A107" s="3" t="s">
         <v>6</v>
       </c>
@@ -1921,45 +1922,45 @@
         <v>5</v>
       </c>
     </row>
-    <row r="108" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A108" s="3" t="s">
         <v>6</v>
       </c>
       <c r="B108" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C108" s="3">
         <v>6</v>
       </c>
     </row>
-    <row r="109" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A109" s="3" t="s">
         <v>6</v>
       </c>
       <c r="B109" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C109" s="3">
         <v>7</v>
       </c>
     </row>
-    <row r="110" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A110" s="3" t="s">
         <v>6</v>
       </c>
       <c r="B110" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C110" s="3">
         <v>8</v>
       </c>
     </row>
-    <row r="111" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A111" s="3" t="s">
         <v>6</v>
       </c>
       <c r="B111" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C111" s="3">
         <v>9</v>
@@ -1970,24 +1971,24 @@
         <v>6</v>
       </c>
       <c r="B112" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C112" s="3">
         <v>10</v>
       </c>
     </row>
-    <row r="113" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A113" s="3" t="s">
         <v>6</v>
       </c>
       <c r="B113" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C113" s="3">
         <v>11</v>
       </c>
     </row>
-    <row r="114" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A114" s="3" t="s">
         <v>6</v>
       </c>
@@ -1998,7 +1999,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="115" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A115" s="3" t="s">
         <v>6</v>
       </c>
@@ -2009,7 +2010,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="116" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A116" s="3" t="s">
         <v>6</v>
       </c>
@@ -2020,7 +2021,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="117" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A117" s="3" t="s">
         <v>6</v>
       </c>
@@ -2031,7 +2032,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="118" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A118" s="3" t="s">
         <v>6</v>
       </c>
@@ -2042,7 +2043,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="119" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A119" s="3" t="s">
         <v>6</v>
       </c>
@@ -2053,7 +2054,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="120" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A120" s="3" t="s">
         <v>6</v>
       </c>
@@ -2064,7 +2065,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="121" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A121" s="3" t="s">
         <v>6</v>
       </c>
@@ -2075,7 +2076,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="122" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A122" s="3" t="s">
         <v>6</v>
       </c>
@@ -2086,7 +2087,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="123" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A123" s="3" t="s">
         <v>6</v>
       </c>
@@ -2097,7 +2098,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="124" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A124" s="3" t="s">
         <v>6</v>
       </c>
@@ -2108,7 +2109,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="125" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A125" s="3" t="s">
         <v>6</v>
       </c>
@@ -2119,29 +2120,29 @@
         <v>17</v>
       </c>
     </row>
-    <row r="126" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A126" s="3" t="s">
         <v>6</v>
       </c>
       <c r="B126" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C126" s="3">
         <v>18</v>
       </c>
     </row>
-    <row r="127" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A127" s="3" t="s">
         <v>6</v>
       </c>
       <c r="B127" s="3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C127" s="3">
         <v>19</v>
       </c>
     </row>
-    <row r="128" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A128" s="5" t="s">
         <v>13</v>
       </c>
@@ -2152,7 +2153,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="129" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A129" s="7" t="s">
         <v>13</v>
       </c>
@@ -2163,18 +2164,18 @@
         <v>2</v>
       </c>
     </row>
-    <row r="130" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A130" s="7" t="s">
         <v>13</v>
       </c>
       <c r="B130" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C130" s="8">
         <v>3</v>
       </c>
     </row>
-    <row r="131" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A131" s="7" t="s">
         <v>13</v>
       </c>
@@ -2185,7 +2186,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="132" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A132" s="7" t="s">
         <v>13</v>
       </c>
@@ -2196,45 +2197,45 @@
         <v>5</v>
       </c>
     </row>
-    <row r="133" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A133" s="7" t="s">
         <v>13</v>
       </c>
       <c r="B133" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C133" s="8">
         <v>6</v>
       </c>
     </row>
-    <row r="134" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A134" s="7" t="s">
         <v>13</v>
       </c>
       <c r="B134" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C134" s="8">
         <v>7</v>
       </c>
     </row>
-    <row r="135" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A135" s="7" t="s">
         <v>13</v>
       </c>
       <c r="B135" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C135" s="8">
         <v>8</v>
       </c>
     </row>
-    <row r="136" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A136" s="7" t="s">
         <v>13</v>
       </c>
       <c r="B136" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C136" s="8">
         <v>9</v>
@@ -2245,24 +2246,24 @@
         <v>13</v>
       </c>
       <c r="B137" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C137" s="8">
         <v>10</v>
       </c>
     </row>
-    <row r="138" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A138" s="7" t="s">
         <v>13</v>
       </c>
       <c r="B138" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C138" s="8">
         <v>11</v>
       </c>
     </row>
-    <row r="139" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A139" s="7" t="s">
         <v>13</v>
       </c>
@@ -2273,7 +2274,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="140" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A140" s="7" t="s">
         <v>13</v>
       </c>
@@ -2284,7 +2285,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="141" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A141" s="7" t="s">
         <v>13</v>
       </c>
@@ -2295,7 +2296,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="142" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A142" s="7" t="s">
         <v>13</v>
       </c>
@@ -2306,7 +2307,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="143" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A143" s="7" t="s">
         <v>13</v>
       </c>
@@ -2317,7 +2318,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="144" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A144" s="7" t="s">
         <v>13</v>
       </c>
@@ -2328,7 +2329,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="145" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A145" s="7" t="s">
         <v>13</v>
       </c>
@@ -2339,7 +2340,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="146" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A146" s="7" t="s">
         <v>13</v>
       </c>
@@ -2350,7 +2351,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="147" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A147" s="7" t="s">
         <v>13</v>
       </c>
@@ -2361,7 +2362,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="148" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A148" s="7" t="s">
         <v>13</v>
       </c>
@@ -2372,7 +2373,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="149" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A149" s="7" t="s">
         <v>13</v>
       </c>
@@ -2383,18 +2384,18 @@
         <v>16</v>
       </c>
     </row>
-    <row r="150" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A150" s="7" t="s">
         <v>13</v>
       </c>
       <c r="B150" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C150" s="8">
         <v>17</v>
       </c>
     </row>
-    <row r="151" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A151" s="7" t="s">
         <v>13</v>
       </c>
@@ -2405,18 +2406,18 @@
         <v>18</v>
       </c>
     </row>
-    <row r="152" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A152" s="7" t="s">
         <v>13</v>
       </c>
       <c r="B152" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C152" s="8">
         <v>19</v>
       </c>
     </row>
-    <row r="153" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A153" s="7" t="s">
         <v>12</v>
       </c>
@@ -2427,18 +2428,18 @@
         <v>1</v>
       </c>
     </row>
-    <row r="154" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A154" s="7" t="s">
         <v>12</v>
       </c>
       <c r="B154" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C154" s="8">
         <v>2</v>
       </c>
     </row>
-    <row r="155" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A155" s="7" t="s">
         <v>12</v>
       </c>
@@ -2449,7 +2450,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="156" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A156" s="7" t="s">
         <v>12</v>
       </c>
@@ -2460,7 +2461,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="157" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A157" s="7" t="s">
         <v>12</v>
       </c>
@@ -2471,45 +2472,45 @@
         <v>5</v>
       </c>
     </row>
-    <row r="158" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A158" s="7" t="s">
         <v>12</v>
       </c>
       <c r="B158" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C158" s="8">
         <v>6</v>
       </c>
     </row>
-    <row r="159" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A159" s="7" t="s">
         <v>12</v>
       </c>
       <c r="B159" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C159" s="8">
         <v>7</v>
       </c>
     </row>
-    <row r="160" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A160" s="7" t="s">
         <v>12</v>
       </c>
       <c r="B160" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C160" s="8">
         <v>8</v>
       </c>
     </row>
-    <row r="161" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A161" s="7" t="s">
         <v>12</v>
       </c>
       <c r="B161" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C161" s="8">
         <v>9</v>
@@ -2520,24 +2521,24 @@
         <v>12</v>
       </c>
       <c r="B162" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C162" s="8">
         <v>10</v>
       </c>
     </row>
-    <row r="163" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A163" s="7" t="s">
         <v>12</v>
       </c>
       <c r="B163" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C163" s="8">
         <v>11</v>
       </c>
     </row>
-    <row r="164" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A164" s="7" t="s">
         <v>12</v>
       </c>
@@ -2548,7 +2549,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="165" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A165" s="7" t="s">
         <v>12</v>
       </c>
@@ -2559,7 +2560,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="166" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A166" s="7" t="s">
         <v>12</v>
       </c>
@@ -2570,7 +2571,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="167" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A167" s="7" t="s">
         <v>12</v>
       </c>
@@ -2581,7 +2582,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="168" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A168" s="7" t="s">
         <v>12</v>
       </c>
@@ -2592,7 +2593,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="169" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A169" s="7" t="s">
         <v>12</v>
       </c>
@@ -2603,7 +2604,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="170" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A170" s="7" t="s">
         <v>12</v>
       </c>
@@ -2614,7 +2615,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="171" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A171" s="7" t="s">
         <v>12</v>
       </c>
@@ -2625,18 +2626,18 @@
         <v>29</v>
       </c>
     </row>
-    <row r="172" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A172" s="7" t="s">
         <v>12</v>
       </c>
       <c r="B172" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C172" s="8">
         <v>14</v>
       </c>
     </row>
-    <row r="173" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A173" s="7" t="s">
         <v>12</v>
       </c>
@@ -2647,7 +2648,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="174" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A174" s="7" t="s">
         <v>12</v>
       </c>
@@ -2658,18 +2659,18 @@
         <v>16</v>
       </c>
     </row>
-    <row r="175" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A175" s="7" t="s">
         <v>12</v>
       </c>
       <c r="B175" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C175" s="8">
         <v>17</v>
       </c>
     </row>
-    <row r="176" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A176" s="7" t="s">
         <v>12</v>
       </c>
@@ -2680,29 +2681,29 @@
         <v>18</v>
       </c>
     </row>
-    <row r="177" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A177" s="7" t="s">
         <v>12</v>
       </c>
       <c r="B177" s="7" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C177" s="8">
         <v>19</v>
       </c>
     </row>
-    <row r="178" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A178" s="7" t="s">
         <v>11</v>
       </c>
       <c r="B178" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C178" s="8">
         <v>1</v>
       </c>
     </row>
-    <row r="179" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A179" s="7" t="s">
         <v>11</v>
       </c>
@@ -2713,29 +2714,29 @@
         <v>2</v>
       </c>
     </row>
-    <row r="180" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A180" s="7" t="s">
         <v>11</v>
       </c>
       <c r="B180" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C180" s="8">
         <v>3</v>
       </c>
     </row>
-    <row r="181" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A181" s="7" t="s">
         <v>11</v>
       </c>
       <c r="B181" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C181" s="8">
         <v>4</v>
       </c>
     </row>
-    <row r="182" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A182" s="7" t="s">
         <v>11</v>
       </c>
@@ -2746,45 +2747,45 @@
         <v>5</v>
       </c>
     </row>
-    <row r="183" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A183" s="7" t="s">
         <v>11</v>
       </c>
       <c r="B183" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C183" s="8">
         <v>6</v>
       </c>
     </row>
-    <row r="184" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A184" s="7" t="s">
         <v>11</v>
       </c>
       <c r="B184" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C184" s="8">
         <v>7</v>
       </c>
     </row>
-    <row r="185" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A185" s="7" t="s">
         <v>11</v>
       </c>
       <c r="B185" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C185" s="8">
         <v>8</v>
       </c>
     </row>
-    <row r="186" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A186" s="7" t="s">
         <v>11</v>
       </c>
       <c r="B186" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C186" s="8">
         <v>9</v>
@@ -2795,24 +2796,24 @@
         <v>11</v>
       </c>
       <c r="B187" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C187" s="8">
         <v>10</v>
       </c>
     </row>
-    <row r="188" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A188" s="7" t="s">
         <v>11</v>
       </c>
       <c r="B188" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C188" s="8">
         <v>11</v>
       </c>
     </row>
-    <row r="189" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A189" s="7" t="s">
         <v>11</v>
       </c>
@@ -2823,7 +2824,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="190" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A190" s="7" t="s">
         <v>11</v>
       </c>
@@ -2834,7 +2835,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="191" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A191" s="7" t="s">
         <v>11</v>
       </c>
@@ -2845,7 +2846,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="192" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A192" s="7" t="s">
         <v>11</v>
       </c>
@@ -2856,7 +2857,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="193" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A193" s="7" t="s">
         <v>11</v>
       </c>
@@ -2867,7 +2868,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="194" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A194" s="7" t="s">
         <v>11</v>
       </c>
@@ -2878,7 +2879,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="195" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A195" s="7" t="s">
         <v>11</v>
       </c>
@@ -2889,7 +2890,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="196" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A196" s="7" t="s">
         <v>11</v>
       </c>
@@ -2900,7 +2901,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="197" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A197" s="7" t="s">
         <v>11</v>
       </c>
@@ -2911,7 +2912,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="198" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A198" s="7" t="s">
         <v>11</v>
       </c>
@@ -2922,29 +2923,29 @@
         <v>15</v>
       </c>
     </row>
-    <row r="199" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A199" s="7" t="s">
         <v>11</v>
       </c>
       <c r="B199" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C199" s="8">
         <v>16</v>
       </c>
     </row>
-    <row r="200" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A200" s="7" t="s">
         <v>11</v>
       </c>
       <c r="B200" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C200" s="8">
         <v>17</v>
       </c>
     </row>
-    <row r="201" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A201" s="7" t="s">
         <v>11</v>
       </c>
@@ -2955,18 +2956,18 @@
         <v>18</v>
       </c>
     </row>
-    <row r="202" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A202" s="7" t="s">
         <v>11</v>
       </c>
       <c r="B202" s="7" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C202" s="8">
         <v>19</v>
       </c>
     </row>
-    <row r="203" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A203" s="7" t="s">
         <v>10</v>
       </c>
@@ -2977,18 +2978,18 @@
         <v>1</v>
       </c>
     </row>
-    <row r="204" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A204" s="7" t="s">
         <v>10</v>
       </c>
       <c r="B204" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C204" s="8">
         <v>2</v>
       </c>
     </row>
-    <row r="205" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A205" s="7" t="s">
         <v>10</v>
       </c>
@@ -2999,7 +3000,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="206" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A206" s="7" t="s">
         <v>10</v>
       </c>
@@ -3010,7 +3011,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="207" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A207" s="7" t="s">
         <v>10</v>
       </c>
@@ -3021,45 +3022,45 @@
         <v>5</v>
       </c>
     </row>
-    <row r="208" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A208" s="7" t="s">
         <v>10</v>
       </c>
       <c r="B208" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C208" s="8">
         <v>6</v>
       </c>
     </row>
-    <row r="209" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A209" s="7" t="s">
         <v>10</v>
       </c>
       <c r="B209" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C209" s="8">
         <v>7</v>
       </c>
     </row>
-    <row r="210" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A210" s="7" t="s">
         <v>10</v>
       </c>
       <c r="B210" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C210" s="8">
         <v>8</v>
       </c>
     </row>
-    <row r="211" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A211" s="7" t="s">
         <v>10</v>
       </c>
       <c r="B211" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C211" s="8">
         <v>9</v>
@@ -3070,24 +3071,24 @@
         <v>10</v>
       </c>
       <c r="B212" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C212" s="8">
         <v>10</v>
       </c>
     </row>
-    <row r="213" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A213" s="7" t="s">
         <v>10</v>
       </c>
       <c r="B213" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C213" s="8">
         <v>11</v>
       </c>
     </row>
-    <row r="214" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A214" s="7" t="s">
         <v>10</v>
       </c>
@@ -3098,7 +3099,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="215" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A215" s="7" t="s">
         <v>10</v>
       </c>
@@ -3109,7 +3110,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="216" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A216" s="7" t="s">
         <v>10</v>
       </c>
@@ -3120,7 +3121,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="217" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A217" s="7" t="s">
         <v>10</v>
       </c>
@@ -3131,7 +3132,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="218" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A218" s="7" t="s">
         <v>10</v>
       </c>
@@ -3142,7 +3143,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="219" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A219" s="7" t="s">
         <v>10</v>
       </c>
@@ -3153,7 +3154,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="220" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A220" s="7" t="s">
         <v>10</v>
       </c>
@@ -3164,7 +3165,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="221" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A221" s="7" t="s">
         <v>10</v>
       </c>
@@ -3175,7 +3176,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="222" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A222" s="7" t="s">
         <v>10</v>
       </c>
@@ -3186,7 +3187,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="223" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A223" s="7" t="s">
         <v>10</v>
       </c>
@@ -3197,7 +3198,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="224" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A224" s="7" t="s">
         <v>10</v>
       </c>
@@ -3208,86 +3209,86 @@
         <v>16</v>
       </c>
     </row>
-    <row r="225" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A225" s="7" t="s">
         <v>10</v>
       </c>
       <c r="B225" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C225" s="8">
         <v>17</v>
       </c>
     </row>
-    <row r="226" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A226" s="7" t="s">
         <v>10</v>
       </c>
       <c r="B226" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C226" s="8">
         <v>18</v>
       </c>
     </row>
-    <row r="227" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A227" s="7" t="s">
         <v>10</v>
       </c>
       <c r="B227" s="7" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C227" s="8">
         <v>19</v>
       </c>
     </row>
-    <row r="228" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A228" s="7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B228" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C228" s="8">
         <v>1</v>
       </c>
     </row>
-    <row r="229" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A229" s="7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B229" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C229" s="8">
         <v>2</v>
       </c>
     </row>
-    <row r="230" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A230" s="7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B230" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C230" s="8">
         <v>3</v>
       </c>
     </row>
-    <row r="231" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A231" s="7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B231" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C231" s="8">
         <v>4</v>
       </c>
     </row>
-    <row r="232" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A232" s="7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B232" s="7" t="s">
         <v>30</v>
@@ -3296,45 +3297,45 @@
         <v>5</v>
       </c>
     </row>
-    <row r="233" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A233" s="7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B233" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C233" s="8">
         <v>6</v>
       </c>
     </row>
-    <row r="234" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A234" s="7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B234" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C234" s="8">
         <v>7</v>
       </c>
     </row>
-    <row r="235" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A235" s="7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B235" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C235" s="8">
         <v>8</v>
       </c>
     </row>
-    <row r="236" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A236" s="7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B236" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C236" s="8">
         <v>9</v>
@@ -3342,29 +3343,29 @@
     </row>
     <row r="237" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A237" s="7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B237" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C237" s="8">
         <v>10</v>
       </c>
     </row>
-    <row r="238" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A238" s="7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B238" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C238" s="8">
         <v>11</v>
       </c>
     </row>
-    <row r="239" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A239" s="7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B239" s="7" t="s">
         <v>20</v>
@@ -3373,9 +3374,9 @@
         <v>12</v>
       </c>
     </row>
-    <row r="240" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A240" s="7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B240" s="3" t="s">
         <v>21</v>
@@ -3384,9 +3385,9 @@
         <v>22</v>
       </c>
     </row>
-    <row r="241" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A241" s="7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B241" s="3" t="s">
         <v>21</v>
@@ -3395,9 +3396,9 @@
         <v>24</v>
       </c>
     </row>
-    <row r="242" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A242" s="7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B242" s="3" t="s">
         <v>23</v>
@@ -3406,9 +3407,9 @@
         <v>25</v>
       </c>
     </row>
-    <row r="243" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A243" s="7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B243" s="3" t="s">
         <v>23</v>
@@ -3417,9 +3418,9 @@
         <v>26</v>
       </c>
     </row>
-    <row r="244" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A244" s="7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B244" s="3" t="s">
         <v>21</v>
@@ -3428,9 +3429,9 @@
         <v>27</v>
       </c>
     </row>
-    <row r="245" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A245" s="7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B245" s="3" t="s">
         <v>23</v>
@@ -3439,9 +3440,9 @@
         <v>28</v>
       </c>
     </row>
-    <row r="246" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A246" s="7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B246" s="3" t="s">
         <v>23</v>
@@ -3450,20 +3451,20 @@
         <v>29</v>
       </c>
     </row>
-    <row r="247" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A247" s="7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B247" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C247" s="8">
         <v>14</v>
       </c>
     </row>
-    <row r="248" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A248" s="7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B248" s="7" t="s">
         <v>30</v>
@@ -3472,9 +3473,9 @@
         <v>15</v>
       </c>
     </row>
-    <row r="249" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A249" s="7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B249" s="7" t="s">
         <v>30</v>
@@ -3483,51 +3484,51 @@
         <v>16</v>
       </c>
     </row>
-    <row r="250" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A250" s="7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B250" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C250" s="8">
         <v>17</v>
       </c>
     </row>
-    <row r="251" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A251" s="7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B251" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C251" s="8">
         <v>18</v>
       </c>
     </row>
-    <row r="252" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A252" s="7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B252" s="7" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C252" s="8">
         <v>19</v>
       </c>
     </row>
-    <row r="253" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A253" s="7" t="s">
         <v>9</v>
       </c>
       <c r="B253" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C253" s="8">
         <v>1</v>
       </c>
     </row>
-    <row r="254" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A254" s="7" t="s">
         <v>9</v>
       </c>
@@ -3538,7 +3539,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="255" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A255" s="7" t="s">
         <v>9</v>
       </c>
@@ -3549,7 +3550,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="256" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A256" s="7" t="s">
         <v>9</v>
       </c>
@@ -3560,7 +3561,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="257" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A257" s="7" t="s">
         <v>9</v>
       </c>
@@ -3571,45 +3572,45 @@
         <v>5</v>
       </c>
     </row>
-    <row r="258" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A258" s="7" t="s">
         <v>9</v>
       </c>
       <c r="B258" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C258" s="8">
         <v>6</v>
       </c>
     </row>
-    <row r="259" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A259" s="7" t="s">
         <v>9</v>
       </c>
       <c r="B259" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C259" s="8">
         <v>7</v>
       </c>
     </row>
-    <row r="260" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A260" s="7" t="s">
         <v>9</v>
       </c>
       <c r="B260" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C260" s="8">
         <v>8</v>
       </c>
     </row>
-    <row r="261" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A261" s="7" t="s">
         <v>9</v>
       </c>
       <c r="B261" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C261" s="8">
         <v>9</v>
@@ -3620,24 +3621,24 @@
         <v>9</v>
       </c>
       <c r="B262" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C262" s="8">
         <v>10</v>
       </c>
     </row>
-    <row r="263" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A263" s="7" t="s">
         <v>9</v>
       </c>
       <c r="B263" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C263" s="8">
         <v>11</v>
       </c>
     </row>
-    <row r="264" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A264" s="7" t="s">
         <v>9</v>
       </c>
@@ -3648,7 +3649,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="265" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A265" s="7" t="s">
         <v>9</v>
       </c>
@@ -3659,7 +3660,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="266" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A266" s="7" t="s">
         <v>9</v>
       </c>
@@ -3670,7 +3671,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="267" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A267" s="7" t="s">
         <v>9</v>
       </c>
@@ -3681,7 +3682,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="268" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A268" s="7" t="s">
         <v>9</v>
       </c>
@@ -3692,7 +3693,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="269" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A269" s="7" t="s">
         <v>9</v>
       </c>
@@ -3703,7 +3704,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="270" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A270" s="7" t="s">
         <v>9</v>
       </c>
@@ -3714,7 +3715,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="271" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A271" s="7" t="s">
         <v>9</v>
       </c>
@@ -3725,7 +3726,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="272" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A272" s="7" t="s">
         <v>9</v>
       </c>
@@ -3736,7 +3737,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="273" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A273" s="7" t="s">
         <v>9</v>
       </c>
@@ -3747,29 +3748,29 @@
         <v>15</v>
       </c>
     </row>
-    <row r="274" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A274" s="7" t="s">
         <v>9</v>
       </c>
       <c r="B274" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C274" s="8">
         <v>16</v>
       </c>
     </row>
-    <row r="275" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A275" s="7" t="s">
         <v>9</v>
       </c>
       <c r="B275" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C275" s="8">
         <v>17</v>
       </c>
     </row>
-    <row r="276" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A276" s="7" t="s">
         <v>9</v>
       </c>
@@ -3780,51 +3781,51 @@
         <v>18</v>
       </c>
     </row>
-    <row r="277" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A277" s="9" t="s">
         <v>9</v>
       </c>
       <c r="B277" s="9" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C277" s="10">
         <v>19</v>
       </c>
     </row>
-    <row r="278" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A278" s="3" t="s">
         <v>2</v>
       </c>
       <c r="B278" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C278" s="3">
         <v>1</v>
       </c>
     </row>
-    <row r="279" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A279" s="3" t="s">
         <v>2</v>
       </c>
       <c r="B279" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C279" s="3">
         <v>2</v>
       </c>
     </row>
-    <row r="280" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A280" s="3" t="s">
         <v>2</v>
       </c>
       <c r="B280" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C280" s="3">
         <v>3</v>
       </c>
     </row>
-    <row r="281" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A281" s="3" t="s">
         <v>2</v>
       </c>
@@ -3835,7 +3836,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="282" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A282" s="3" t="s">
         <v>2</v>
       </c>
@@ -3846,45 +3847,45 @@
         <v>5</v>
       </c>
     </row>
-    <row r="283" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A283" s="3" t="s">
         <v>2</v>
       </c>
       <c r="B283" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C283" s="3">
         <v>6</v>
       </c>
     </row>
-    <row r="284" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A284" s="3" t="s">
         <v>2</v>
       </c>
       <c r="B284" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C284" s="3">
         <v>7</v>
       </c>
     </row>
-    <row r="285" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A285" s="3" t="s">
         <v>2</v>
       </c>
       <c r="B285" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C285" s="3">
         <v>8</v>
       </c>
     </row>
-    <row r="286" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A286" s="3" t="s">
         <v>2</v>
       </c>
       <c r="B286" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C286" s="3">
         <v>9</v>
@@ -3895,24 +3896,24 @@
         <v>2</v>
       </c>
       <c r="B287" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C287" s="3">
         <v>10</v>
       </c>
     </row>
-    <row r="288" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A288" s="3" t="s">
         <v>2</v>
       </c>
       <c r="B288" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C288" s="3">
         <v>11</v>
       </c>
     </row>
-    <row r="289" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A289" s="3" t="s">
         <v>2</v>
       </c>
@@ -3923,7 +3924,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="290" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A290" s="3" t="s">
         <v>2</v>
       </c>
@@ -3934,7 +3935,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="291" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A291" s="3" t="s">
         <v>2</v>
       </c>
@@ -3945,7 +3946,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="292" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A292" s="3" t="s">
         <v>2</v>
       </c>
@@ -3956,7 +3957,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="293" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A293" s="3" t="s">
         <v>2</v>
       </c>
@@ -3967,7 +3968,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="294" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A294" s="3" t="s">
         <v>2</v>
       </c>
@@ -3979,7 +3980,7 @@
       </c>
       <c r="G294" s="4"/>
     </row>
-    <row r="295" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A295" s="3" t="s">
         <v>2</v>
       </c>
@@ -3990,7 +3991,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="296" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A296" s="3" t="s">
         <v>2</v>
       </c>
@@ -4001,18 +4002,18 @@
         <v>29</v>
       </c>
     </row>
-    <row r="297" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A297" s="3" t="s">
         <v>2</v>
       </c>
       <c r="B297" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C297" s="3">
         <v>14</v>
       </c>
     </row>
-    <row r="298" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A298" s="3" t="s">
         <v>2</v>
       </c>
@@ -4023,7 +4024,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="299" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A299" s="3" t="s">
         <v>2</v>
       </c>
@@ -4034,40 +4035,40 @@
         <v>16</v>
       </c>
     </row>
-    <row r="300" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A300" s="3" t="s">
         <v>2</v>
       </c>
       <c r="B300" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C300" s="3">
         <v>17</v>
       </c>
     </row>
-    <row r="301" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A301" s="3" t="s">
         <v>2</v>
       </c>
       <c r="B301" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C301" s="3">
         <v>18</v>
       </c>
     </row>
-    <row r="302" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A302" s="3" t="s">
         <v>2</v>
       </c>
       <c r="B302" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C302" s="3">
         <v>19</v>
       </c>
     </row>
-    <row r="303" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A303" s="3" t="s">
         <v>18</v>
       </c>
@@ -4078,7 +4079,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="304" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A304" s="3" t="s">
         <v>18</v>
       </c>
@@ -4089,7 +4090,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="305" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A305" s="3" t="s">
         <v>18</v>
       </c>
@@ -4100,7 +4101,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="306" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A306" s="3" t="s">
         <v>18</v>
       </c>
@@ -4111,7 +4112,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="307" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A307" s="3" t="s">
         <v>18</v>
       </c>
@@ -4122,45 +4123,45 @@
         <v>5</v>
       </c>
     </row>
-    <row r="308" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A308" s="3" t="s">
         <v>18</v>
       </c>
       <c r="B308" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C308" s="3">
         <v>6</v>
       </c>
     </row>
-    <row r="309" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A309" s="3" t="s">
         <v>18</v>
       </c>
       <c r="B309" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C309" s="3">
         <v>7</v>
       </c>
     </row>
-    <row r="310" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="310" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A310" s="3" t="s">
         <v>18</v>
       </c>
       <c r="B310" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C310" s="3">
         <v>8</v>
       </c>
     </row>
-    <row r="311" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="311" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A311" s="3" t="s">
         <v>18</v>
       </c>
       <c r="B311" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C311" s="3">
         <v>9</v>
@@ -4171,24 +4172,24 @@
         <v>18</v>
       </c>
       <c r="B312" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C312" s="3">
         <v>10</v>
       </c>
     </row>
-    <row r="313" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="313" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A313" s="3" t="s">
         <v>18</v>
       </c>
       <c r="B313" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C313" s="3">
         <v>11</v>
       </c>
     </row>
-    <row r="314" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="314" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A314" s="3" t="s">
         <v>18</v>
       </c>
@@ -4199,7 +4200,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="315" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="315" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A315" s="3" t="s">
         <v>18</v>
       </c>
@@ -4210,7 +4211,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="316" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="316" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A316" s="3" t="s">
         <v>18</v>
       </c>
@@ -4221,7 +4222,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="317" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="317" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A317" s="3" t="s">
         <v>18</v>
       </c>
@@ -4232,7 +4233,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="318" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="318" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A318" s="3" t="s">
         <v>18</v>
       </c>
@@ -4243,7 +4244,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="319" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="319" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A319" s="3" t="s">
         <v>18</v>
       </c>
@@ -4254,7 +4255,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="320" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="320" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A320" s="3" t="s">
         <v>18</v>
       </c>
@@ -4265,7 +4266,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="321" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="321" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A321" s="3" t="s">
         <v>18</v>
       </c>
@@ -4276,18 +4277,18 @@
         <v>29</v>
       </c>
     </row>
-    <row r="322" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="322" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A322" s="3" t="s">
         <v>18</v>
       </c>
       <c r="B322" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C322" s="3">
         <v>14</v>
       </c>
     </row>
-    <row r="323" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="323" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A323" s="3" t="s">
         <v>18</v>
       </c>
@@ -4298,7 +4299,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="324" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="324" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A324" s="3" t="s">
         <v>18</v>
       </c>
@@ -4309,18 +4310,18 @@
         <v>16</v>
       </c>
     </row>
-    <row r="325" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="325" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A325" s="3" t="s">
         <v>18</v>
       </c>
       <c r="B325" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C325" s="3">
         <v>17</v>
       </c>
     </row>
-    <row r="326" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="326" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A326" s="3" t="s">
         <v>18</v>
       </c>
@@ -4331,18 +4332,18 @@
         <v>18</v>
       </c>
     </row>
-    <row r="327" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="327" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A327" s="3" t="s">
         <v>18</v>
       </c>
       <c r="B327" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C327" s="3">
         <v>19</v>
       </c>
     </row>
-    <row r="328" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="328" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A328" s="3" t="s">
         <v>15</v>
       </c>
@@ -4353,40 +4354,40 @@
         <v>1</v>
       </c>
     </row>
-    <row r="329" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="329" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A329" s="3" t="s">
         <v>15</v>
       </c>
       <c r="B329" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C329" s="3">
         <v>2</v>
       </c>
     </row>
-    <row r="330" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="330" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A330" s="3" t="s">
         <v>15</v>
       </c>
       <c r="B330" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C330" s="3">
         <v>3</v>
       </c>
     </row>
-    <row r="331" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="331" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A331" s="3" t="s">
         <v>15</v>
       </c>
       <c r="B331" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C331" s="3">
         <v>4</v>
       </c>
     </row>
-    <row r="332" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="332" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A332" s="3" t="s">
         <v>15</v>
       </c>
@@ -4397,45 +4398,45 @@
         <v>5</v>
       </c>
     </row>
-    <row r="333" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="333" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A333" s="3" t="s">
         <v>15</v>
       </c>
       <c r="B333" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C333" s="3">
         <v>6</v>
       </c>
     </row>
-    <row r="334" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="334" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A334" s="3" t="s">
         <v>15</v>
       </c>
       <c r="B334" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C334" s="3">
         <v>7</v>
       </c>
     </row>
-    <row r="335" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="335" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A335" s="3" t="s">
         <v>15</v>
       </c>
       <c r="B335" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C335" s="3">
         <v>8</v>
       </c>
     </row>
-    <row r="336" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="336" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A336" s="3" t="s">
         <v>15</v>
       </c>
       <c r="B336" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C336" s="3">
         <v>9</v>
@@ -4446,24 +4447,24 @@
         <v>15</v>
       </c>
       <c r="B337" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C337" s="3">
         <v>10</v>
       </c>
     </row>
-    <row r="338" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="338" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A338" s="3" t="s">
         <v>15</v>
       </c>
       <c r="B338" s="3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C338" s="3">
         <v>11</v>
       </c>
     </row>
-    <row r="339" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="339" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A339" s="3" t="s">
         <v>15</v>
       </c>
@@ -4474,7 +4475,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="340" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="340" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A340" s="3" t="s">
         <v>15</v>
       </c>
@@ -4485,7 +4486,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="341" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="341" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A341" s="3" t="s">
         <v>15</v>
       </c>
@@ -4496,7 +4497,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="342" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="342" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A342" s="3" t="s">
         <v>15</v>
       </c>
@@ -4507,7 +4508,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="343" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="343" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A343" s="3" t="s">
         <v>15</v>
       </c>
@@ -4518,7 +4519,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="344" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="344" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A344" s="3" t="s">
         <v>15</v>
       </c>
@@ -4529,7 +4530,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="345" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="345" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A345" s="3" t="s">
         <v>15</v>
       </c>
@@ -4540,7 +4541,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="346" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="346" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A346" s="3" t="s">
         <v>15</v>
       </c>
@@ -4551,7 +4552,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="347" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="347" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A347" s="3" t="s">
         <v>15</v>
       </c>
@@ -4562,7 +4563,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="348" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="348" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A348" s="3" t="s">
         <v>15</v>
       </c>
@@ -4573,7 +4574,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="349" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="349" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A349" s="3" t="s">
         <v>15</v>
       </c>
@@ -4584,73 +4585,73 @@
         <v>16</v>
       </c>
     </row>
-    <row r="350" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="350" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A350" s="3" t="s">
         <v>15</v>
       </c>
       <c r="B350" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C350" s="3">
         <v>17</v>
       </c>
     </row>
-    <row r="351" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="351" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A351" s="3" t="s">
         <v>15</v>
       </c>
       <c r="B351" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C351" s="3">
         <v>18</v>
       </c>
     </row>
-    <row r="352" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="352" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A352" s="3" t="s">
         <v>15</v>
       </c>
       <c r="B352" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C352" s="3">
         <v>19</v>
       </c>
     </row>
-    <row r="353" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="353" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A353" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B353" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C353" s="3">
         <v>1</v>
       </c>
     </row>
-    <row r="354" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="354" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A354" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B354" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C354" s="3">
         <v>2</v>
       </c>
     </row>
-    <row r="355" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="355" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A355" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B355" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C355" s="3">
         <v>3</v>
       </c>
     </row>
-    <row r="356" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="356" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A356" s="3" t="s">
         <v>7</v>
       </c>
@@ -4661,7 +4662,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="357" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="357" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A357" s="3" t="s">
         <v>7</v>
       </c>
@@ -4672,45 +4673,45 @@
         <v>5</v>
       </c>
     </row>
-    <row r="358" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="358" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A358" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B358" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C358" s="3">
         <v>6</v>
       </c>
     </row>
-    <row r="359" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="359" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A359" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B359" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C359" s="3">
         <v>7</v>
       </c>
     </row>
-    <row r="360" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="360" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A360" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B360" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C360" s="3">
         <v>8</v>
       </c>
     </row>
-    <row r="361" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="361" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A361" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B361" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C361" s="3">
         <v>9</v>
@@ -4721,24 +4722,24 @@
         <v>7</v>
       </c>
       <c r="B362" s="3" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C362" s="3">
         <v>10</v>
       </c>
     </row>
-    <row r="363" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="363" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A363" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B363" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C363" s="3">
         <v>11</v>
       </c>
     </row>
-    <row r="364" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="364" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A364" s="3" t="s">
         <v>7</v>
       </c>
@@ -4749,7 +4750,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="365" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="365" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A365" s="3" t="s">
         <v>7</v>
       </c>
@@ -4760,7 +4761,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="366" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="366" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A366" s="3" t="s">
         <v>7</v>
       </c>
@@ -4771,7 +4772,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="367" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="367" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A367" s="3" t="s">
         <v>7</v>
       </c>
@@ -4782,7 +4783,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="368" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="368" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A368" s="3" t="s">
         <v>7</v>
       </c>
@@ -4793,7 +4794,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="369" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="369" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A369" s="3" t="s">
         <v>7</v>
       </c>
@@ -4804,7 +4805,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="370" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="370" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A370" s="3" t="s">
         <v>7</v>
       </c>
@@ -4815,7 +4816,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="371" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="371" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A371" s="3" t="s">
         <v>7</v>
       </c>
@@ -4826,18 +4827,18 @@
         <v>29</v>
       </c>
     </row>
-    <row r="372" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="372" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A372" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B372" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C372" s="3">
         <v>14</v>
       </c>
     </row>
-    <row r="373" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="373" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A373" s="3" t="s">
         <v>7</v>
       </c>
@@ -4848,84 +4849,84 @@
         <v>15</v>
       </c>
     </row>
-    <row r="374" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="374" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A374" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B374" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C374" s="3">
         <v>16</v>
       </c>
     </row>
-    <row r="375" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="375" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A375" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B375" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C375" s="3">
         <v>17</v>
       </c>
     </row>
-    <row r="376" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="376" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A376" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B376" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C376" s="3">
         <v>18</v>
       </c>
     </row>
-    <row r="377" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="377" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A377" s="3" t="s">
         <v>7</v>
       </c>
       <c r="B377" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C377" s="3">
         <v>19</v>
       </c>
     </row>
-    <row r="378" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="378" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A378" s="3" t="s">
         <v>14</v>
       </c>
       <c r="B378" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C378" s="3">
         <v>1</v>
       </c>
     </row>
-    <row r="379" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="379" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A379" s="3" t="s">
         <v>14</v>
       </c>
       <c r="B379" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C379" s="3">
         <v>2</v>
       </c>
     </row>
-    <row r="380" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="380" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A380" s="3" t="s">
         <v>14</v>
       </c>
       <c r="B380" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C380" s="3">
         <v>3</v>
       </c>
     </row>
-    <row r="381" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="381" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A381" s="3" t="s">
         <v>14</v>
       </c>
@@ -4936,7 +4937,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="382" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="382" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A382" s="3" t="s">
         <v>14</v>
       </c>
@@ -4947,45 +4948,45 @@
         <v>5</v>
       </c>
     </row>
-    <row r="383" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="383" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A383" s="3" t="s">
         <v>14</v>
       </c>
       <c r="B383" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C383" s="3">
         <v>6</v>
       </c>
     </row>
-    <row r="384" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="384" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A384" s="3" t="s">
         <v>14</v>
       </c>
       <c r="B384" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C384" s="3">
         <v>7</v>
       </c>
     </row>
-    <row r="385" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="385" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A385" s="3" t="s">
         <v>14</v>
       </c>
       <c r="B385" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C385" s="3">
         <v>8</v>
       </c>
     </row>
-    <row r="386" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="386" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A386" s="3" t="s">
         <v>14</v>
       </c>
       <c r="B386" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C386" s="3">
         <v>9</v>
@@ -4996,24 +4997,24 @@
         <v>14</v>
       </c>
       <c r="B387" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C387" s="3">
         <v>10</v>
       </c>
     </row>
-    <row r="388" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="388" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A388" s="3" t="s">
         <v>14</v>
       </c>
       <c r="B388" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C388" s="3">
         <v>11</v>
       </c>
     </row>
-    <row r="389" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="389" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A389" s="3" t="s">
         <v>14</v>
       </c>
@@ -5024,7 +5025,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="390" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="390" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A390" s="3" t="s">
         <v>14</v>
       </c>
@@ -5035,7 +5036,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="391" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="391" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A391" s="3" t="s">
         <v>14</v>
       </c>
@@ -5046,7 +5047,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="392" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="392" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A392" s="3" t="s">
         <v>14</v>
       </c>
@@ -5057,7 +5058,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="393" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="393" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A393" s="3" t="s">
         <v>14</v>
       </c>
@@ -5068,7 +5069,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="394" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="394" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A394" s="3" t="s">
         <v>14</v>
       </c>
@@ -5079,7 +5080,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="395" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="395" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A395" s="3" t="s">
         <v>14</v>
       </c>
@@ -5090,7 +5091,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="396" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="396" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A396" s="3" t="s">
         <v>14</v>
       </c>
@@ -5101,73 +5102,73 @@
         <v>29</v>
       </c>
     </row>
-    <row r="397" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="397" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A397" s="3" t="s">
         <v>14</v>
       </c>
       <c r="B397" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C397" s="3">
         <v>14</v>
       </c>
     </row>
-    <row r="398" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="398" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A398" s="3" t="s">
         <v>14</v>
       </c>
       <c r="B398" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C398" s="3">
         <v>15</v>
       </c>
     </row>
-    <row r="399" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="399" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A399" s="3" t="s">
         <v>14</v>
       </c>
       <c r="B399" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C399" s="3">
         <v>16</v>
       </c>
     </row>
-    <row r="400" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="400" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A400" s="3" t="s">
         <v>14</v>
       </c>
       <c r="B400" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C400" s="3">
         <v>17</v>
       </c>
     </row>
-    <row r="401" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="401" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A401" s="3" t="s">
         <v>14</v>
       </c>
       <c r="B401" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C401" s="3">
         <v>18</v>
       </c>
     </row>
-    <row r="402" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="402" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A402" s="3" t="s">
         <v>14</v>
       </c>
       <c r="B402" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C402" s="3">
         <v>19</v>
       </c>
     </row>
-    <row r="403" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="403" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A403" s="3" t="s">
         <v>8</v>
       </c>
@@ -5178,29 +5179,29 @@
         <v>1</v>
       </c>
     </row>
-    <row r="404" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="404" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A404" s="3" t="s">
         <v>8</v>
       </c>
       <c r="B404" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C404" s="3">
         <v>2</v>
       </c>
     </row>
-    <row r="405" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="405" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A405" s="3" t="s">
         <v>8</v>
       </c>
       <c r="B405" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C405" s="3">
         <v>3</v>
       </c>
     </row>
-    <row r="406" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="406" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A406" s="3" t="s">
         <v>8</v>
       </c>
@@ -5211,7 +5212,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="407" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="407" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A407" s="3" t="s">
         <v>8</v>
       </c>
@@ -5222,45 +5223,45 @@
         <v>5</v>
       </c>
     </row>
-    <row r="408" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="408" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A408" s="3" t="s">
         <v>8</v>
       </c>
       <c r="B408" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C408" s="3">
         <v>6</v>
       </c>
     </row>
-    <row r="409" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="409" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A409" s="3" t="s">
         <v>8</v>
       </c>
       <c r="B409" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C409" s="3">
         <v>7</v>
       </c>
     </row>
-    <row r="410" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="410" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A410" s="3" t="s">
         <v>8</v>
       </c>
       <c r="B410" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C410" s="3">
         <v>8</v>
       </c>
     </row>
-    <row r="411" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="411" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A411" s="3" t="s">
         <v>8</v>
       </c>
       <c r="B411" s="3" t="s">
-        <v>23</v>
+        <v>34</v>
       </c>
       <c r="C411" s="3">
         <v>9</v>
@@ -5271,24 +5272,24 @@
         <v>8</v>
       </c>
       <c r="B412" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C412" s="3">
         <v>10</v>
       </c>
     </row>
-    <row r="413" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="413" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A413" s="3" t="s">
         <v>8</v>
       </c>
       <c r="B413" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C413" s="3">
         <v>11</v>
       </c>
     </row>
-    <row r="414" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="414" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A414" s="3" t="s">
         <v>8</v>
       </c>
@@ -5299,7 +5300,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="415" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="415" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A415" s="3" t="s">
         <v>8</v>
       </c>
@@ -5310,7 +5311,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="416" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="416" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A416" s="3" t="s">
         <v>8</v>
       </c>
@@ -5321,7 +5322,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="417" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="417" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A417" s="3" t="s">
         <v>8</v>
       </c>
@@ -5332,7 +5333,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="418" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="418" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A418" s="3" t="s">
         <v>8</v>
       </c>
@@ -5343,7 +5344,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="419" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="419" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A419" s="3" t="s">
         <v>8</v>
       </c>
@@ -5354,7 +5355,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="420" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="420" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A420" s="3" t="s">
         <v>8</v>
       </c>
@@ -5365,7 +5366,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="421" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="421" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A421" s="3" t="s">
         <v>8</v>
       </c>
@@ -5376,7 +5377,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="422" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="422" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A422" s="3" t="s">
         <v>8</v>
       </c>
@@ -5387,7 +5388,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="423" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="423" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A423" s="3" t="s">
         <v>8</v>
       </c>
@@ -5398,18 +5399,18 @@
         <v>15</v>
       </c>
     </row>
-    <row r="424" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="424" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A424" s="3" t="s">
         <v>8</v>
       </c>
       <c r="B424" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C424" s="3">
         <v>16</v>
       </c>
     </row>
-    <row r="425" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="425" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A425" s="3" t="s">
         <v>8</v>
       </c>
@@ -5420,7 +5421,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="426" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="426" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A426" s="3" t="s">
         <v>8</v>
       </c>
@@ -5431,12 +5432,12 @@
         <v>18</v>
       </c>
     </row>
-    <row r="427" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="427" spans="1:3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A427" s="3" t="s">
         <v>8</v>
       </c>
       <c r="B427" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C427" s="3">
         <v>19</v>
@@ -5985,6 +5986,13 @@
       <c r="B651" s="12"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:C427" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="2">
+      <filters>
+        <filter val="10"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>